<commit_message>
Add Modules 2–6: 45 notebooks, five practice Sheets, sample district data, live NASA POWER/ERA5 loaders, tests
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FvEzaKk5xvfed5Uezs2t6g
</commit_message>
<xml_diff>
--- a/sheets/WDL_M1_practice.xlsx
+++ b/sheets/WDL_M1_practice.xlsx
@@ -1010,11 +1010,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="52393931"/>
-        <c:axId val="88516942"/>
+        <c:axId val="8087858"/>
+        <c:axId val="49376868"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="52393931"/>
+        <c:axId val="8087858"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1046,7 +1046,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="88516942"/>
+        <c:crossAx val="49376868"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1054,7 +1054,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="88516942"/>
+        <c:axId val="49376868"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1130,7 +1130,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="52393931"/>
+        <c:crossAx val="8087858"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1438,11 +1438,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="26416284"/>
-        <c:axId val="44504194"/>
+        <c:axId val="6460968"/>
+        <c:axId val="73648720"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="26416284"/>
+        <c:axId val="6460968"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1474,7 +1474,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="44504194"/>
+        <c:crossAx val="73648720"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1482,7 +1482,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="44504194"/>
+        <c:axId val="73648720"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1558,7 +1558,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="26416284"/>
+        <c:crossAx val="6460968"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1700,11 +1700,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="47676215"/>
-        <c:axId val="16088938"/>
+        <c:axId val="87653231"/>
+        <c:axId val="31913414"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="47676215"/>
+        <c:axId val="87653231"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1736,7 +1736,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="16088938"/>
+        <c:crossAx val="31913414"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1744,7 +1744,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="16088938"/>
+        <c:axId val="31913414"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1786,7 +1786,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="47676215"/>
+        <c:crossAx val="87653231"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>